<commit_message>
Rename brand to Reserve Clinic and add minimal logo
Renames the concept from the AminoLord working name to Reserve Clinic / ReserveClinic.com across
deliverables and build scripts, renames the deliverable files, adds a vector logo (serif R in a brass
ring with tracked wordmark) with SVG/PNG exports in outputs/brand, places it on both PDF covers and
the brief footer, and records the naming and trademark implications for counsel. Research files keep
the earlier working name; research/README_RENAME.md explains why.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012mqgHCHaCUnT6CFfSB2Ugk
</commit_message>
<xml_diff>
--- a/outputs/03_Peptide_Product_and_Pricing_Audit.xlsx
+++ b/outputs/03_Peptide_Product_and_Pricing_Audit.xlsx
@@ -17756,7 +17756,7 @@
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>AminoLord recommendation [SR]</t>
+          <t>Reserve Clinic recommendation [SR]</t>
         </is>
       </c>
     </row>
@@ -18042,7 +18042,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Model in 07_AminoLord_Financial_Model.xlsx</t>
+          <t>Model in 07_ReserveClinic_Financial_Model.xlsx</t>
         </is>
       </c>
     </row>
@@ -18091,7 +18091,7 @@
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>AminoLord copy rule [SR]</t>
+          <t>Reserve Clinic copy rule [SR]</t>
         </is>
       </c>
     </row>

</xml_diff>